<commit_message>
Tuerchen 24: Breite dreifach, Hoehe gleich; Gesamtplan aktualisiert
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VqGSRUdcAYrcRp9bP6axqV
</commit_message>
<xml_diff>
--- a/10_Aufbereitet/Adventskalender-Gesamtplan.xlsx
+++ b/10_Aufbereitet/Adventskalender-Gesamtplan.xlsx
@@ -1322,7 +1322,7 @@
     <t xml:space="preserve">Türchen 24: Breite und Höhe dreifach oder Fläche dreifach?</t>
   </si>
   <si>
-    <t xml:space="preserve">Breite dreifach. Höhe: Claude lässt sie wie bisher proportional (quadratisch), bitte bestätigen.</t>
+    <t xml:space="preserve">Breite dreifach, Höhe gleich wie die anderen Türchen (Jannik, 24.10.).</t>
   </si>
   <si>
     <t xml:space="preserve">Videoformat des Kalenders: 16:9?</t>
@@ -9614,7 +9614,7 @@
         <v>429</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="10" t="n">
         <v>15</v>
       </c>

</xml_diff>